<commit_message>
Update candidate stash Excel template
</commit_message>
<xml_diff>
--- a/TEMPLATE/(Han.A)Template(ver.0.0.0).xlsx
+++ b/TEMPLATE/(Han.A)Template(ver.0.0.0).xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\윤대영\Desktop\한아\TEMPLATE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TEST\HAN.A\TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79D1D51D-C108-4F60-A915-A7EB4AC40A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16E502AE-C289-4A52-A40F-804317E7FB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45525" yWindow="2160" windowWidth="19200" windowHeight="11265" xr2:uid="{C75FE9E0-A7F3-484F-B9F2-46A99887CF73}"/>
+    <workbookView xWindow="42540" yWindow="3150" windowWidth="19200" windowHeight="11265" activeTab="3" xr2:uid="{C75FE9E0-A7F3-484F-B9F2-46A99887CF73}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA" sheetId="4" r:id="rId1"/>
     <sheet name="예시" sheetId="1" r:id="rId2"/>
     <sheet name="Infos" sheetId="5" r:id="rId3"/>
+    <sheet name="Meta" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -168,7 +169,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{1960067F-F7F8-41C2-B192-60404CBC3A85}">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{E34440B0-C049-45E2-8F6E-ABBB8F8EE9F6}">
       <text>
         <r>
           <rPr>
@@ -179,47 +180,31 @@
             <family val="3"/>
             <charset val="129"/>
           </rPr>
-          <t xml:space="preserve">사이즈가 공란이면 전체 수량으로 간주.
+          <t>윤대영</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{E34440B0-C049-45E2-8F6E-ABBB8F8EE9F6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="돋움"/>
-            <family val="3"/>
-            <charset val="129"/>
-          </rPr>
-          <t>윤대영</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{94CAED08-9514-462A-8E3E-A498A560C4A2}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{94CAED08-9514-462A-8E3E-A498A560C4A2}">
       <text>
         <r>
           <rPr>
@@ -391,7 +376,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{04E3CD5E-2EC1-4059-BD28-BAE97A632CC7}">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{C8DD38D6-B2C7-4F5D-8F71-1B8B75E59A8B}">
       <text>
         <r>
           <rPr>
@@ -402,47 +387,31 @@
             <family val="3"/>
             <charset val="129"/>
           </rPr>
-          <t xml:space="preserve">사이즈가 공란이면 전체 수량으로 간주.
+          <t>윤대영</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{C8DD38D6-B2C7-4F5D-8F71-1B8B75E59A8B}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="돋움"/>
-            <family val="3"/>
-            <charset val="129"/>
-          </rPr>
-          <t>윤대영</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{BF1E74CF-0FF4-41F9-A83E-FCCE26A26E71}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{BF1E74CF-0FF4-41F9-A83E-FCCE26A26E71}">
       <text>
         <r>
           <rPr>
@@ -482,7 +451,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t>상품 코드</t>
   </si>
@@ -542,11 +511,27 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>사이즈</t>
+    <t>interger</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>interger</t>
+    <t>Value</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Key</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Version</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.0.0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LastUpdatedAt</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -657,7 +642,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -673,10 +658,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -706,13 +688,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>495300</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -894,7 +876,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1036,7 +1018,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1130,13 +1112,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>584200</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1531,15 +1513,15 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="4"/>
     <col min="2" max="3" width="9.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="15.75" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.75" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -1549,20 +1531,16 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>16</v>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1573,16 +1551,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6370B8-4E78-42A6-9991-34D40D2A92F1}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="4"/>
     <col min="2" max="3" width="9.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.75" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="15.75" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.75" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -1592,17 +1569,14 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>16</v>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
@@ -1612,13 +1586,10 @@
       <c r="C2" s="4">
         <v>34200</v>
       </c>
-      <c r="D2" s="6">
-        <v>255</v>
+      <c r="D2" s="2">
+        <v>46149</v>
       </c>
       <c r="E2" s="2">
-        <v>46149</v>
-      </c>
-      <c r="F2" s="2">
         <v>46333</v>
       </c>
     </row>
@@ -1635,7 +1606,7 @@
   <sheetPr>
     <tabColor theme="1"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.75" bestFit="1" customWidth="1"/>
@@ -1670,31 +1641,65 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CB963EF-63C1-4F56-A321-066757DDF9FA}">
+  <sheetPr>
+    <tabColor theme="1"/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.08203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>